<commit_message>
Use numbers instead of formatted string
</commit_message>
<xml_diff>
--- a/api/templates/device_utilization/en.xlsx
+++ b/api/templates/device_utilization/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="21126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24931"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\ubuntu\aspect\api\templates\device_utilization\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\stefan\aspect\api\templates\device_utilization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA6904D-1765-4F4F-8EC1-21127141713F}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FB80D8D-D791-4D9C-9C8D-E52862162874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35570" yWindow="1330" windowWidth="22990" windowHeight="16080" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1509" yWindow="746" windowWidth="25945" windowHeight="17768" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Utilization Rate" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -84,6 +84,13 @@
       <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -123,7 +130,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="43">
+  <cellStyleXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -167,15 +174,17 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="43" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="43">
+  <cellStyles count="44">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -219,6 +228,7 @@
     <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="43" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
@@ -556,45 +566,45 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="31.83203125" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:1" ht="20.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A5" s="1"/>
     </row>
-    <row r="6" spans="1:1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:1" ht="16.3" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
[feat/HD-15447] Fixed "Device average utilization per month" report templates
</commit_message>
<xml_diff>
--- a/api/templates/device_utilization/en.xlsx
+++ b/api/templates/device_utilization/en.xlsx
@@ -1,21 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10309"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect-2\api\templates\device_utilization\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/device_utilization/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D354144C-9BB6-FA41-B306-2D81F780EF2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Utilization Rate" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -53,7 +65,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -99,7 +111,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -122,21 +134,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -167,7 +191,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -513,53 +537,50 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.8984375" customWidth="1"/>
+    <col min="1" max="1" width="31.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[feat/HD-15426-Myanmar-update-For-Device-Utilization-rate] Added legend to excel templates
</commit_message>
<xml_diff>
--- a/api/templates/device_utilization/en.xlsx
+++ b/api/templates/device_utilization/en.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10608"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect-2\api\templates\device_utilization\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/device_utilization/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1FB9D02-8537-7A47-BEEE-5302290BCA0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Utilization Rate" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Device Utilization Rate</t>
   </si>
@@ -48,12 +49,15 @@
   </si>
   <si>
     <t>&lt;name&gt;</t>
+  </si>
+  <si>
+    <t>Device percentages are not weighted by their capacity. Therefore, the simple average of these values may differ from the total percentage shown in the system.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -127,16 +131,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -167,7 +172,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -513,57 +518,80 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.8984375" customWidth="1"/>
+    <col min="1" max="1" width="31.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="C2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+    </row>
+    <row r="5" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C2:I4"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
[feat/HD-15426-Myanmar-update-For-Device-Utilization-rate] Added daily capacity column
</commit_message>
<xml_diff>
--- a/api/templates/device_utilization/en.xlsx
+++ b/api/templates/device_utilization/en.xlsx
@@ -8,15 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/device_utilization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1FB9D02-8537-7A47-BEEE-5302290BCA0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72224212-388E-EE4B-8262-8FC9D61CB82D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Utilization Rate" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -25,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Device Utilization Rate</t>
   </si>
@@ -52,6 +63,12 @@
   </si>
   <si>
     <t>Device percentages are not weighted by their capacity. Therefore, the simple average of these values may differ from the total percentage shown in the system.</t>
+  </si>
+  <si>
+    <t>Daily Capacity</t>
+  </si>
+  <si>
+    <t>&lt;dailyTestCapacity&gt;</t>
   </si>
 </sst>
 </file>
@@ -131,7 +148,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -142,6 +159,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,6 +544,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
@@ -573,19 +595,25 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>